<commit_message>
v12.1.0: four regenerated sample files, previews re-rendered to match
Opportunities_SAMPLE.xlsx, CTC_Events_SAMPLE.xlsx and both Portland issue
files replace the hosted copies at the same paths and names. The
opportunities workbook no longer carries a Status or a Last used column, so
the excerpt on the Newsletter page drops its Status column. The events
workbook now flags a missing end time in Missing Info and notes where a map
link does not apply. The Portland issue's Upcoming Events are in date order.

Preview shows a render of the very file Download hands over, so the page
images and the opened-in-Excel and opened-in-Word captures for those three
files were re-taken from the new files. Page counts are unchanged; only the
opportunities sheet's height moved in DIMS.

The ctc-newsletter label stays at v2.0.0 because the hosted zip is v2.0.0.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/samples/CTC_Events_SAMPLE.xlsx
+++ b/downloads/samples/CTC_Events_SAMPLE.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBCB"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,12 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -642,7 +650,7 @@
           <t>18:00</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/example-mass-timber</t>
@@ -703,7 +711,11 @@
           <t>registry</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1136,7 +1148,7 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>https://example.org/eastside-greenway-ride</t>
@@ -1197,7 +1209,11 @@
           <t>registry</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>End Time</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1494,7 +1510,11 @@
           <t>Southeast</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>n/a (address withheld)</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Site Tour</t>
@@ -1905,7 +1925,11 @@
           <t>Online</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>n/a (online)</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Panel Session, Webinar</t>
@@ -1946,7 +1970,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2029,7 +2053,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2112,7 +2136,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2195,7 +2219,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">

</xml_diff>